<commit_message>
Ultrasonic sensor code working on the STM32 with custom LCD driver
</commit_message>
<xml_diff>
--- a/PCB/JAARK_PCB_MOTOR/JAARK_PCB_MOTOR.xlsx
+++ b/PCB/JAARK_PCB_MOTOR/JAARK_PCB_MOTOR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonar\JAARK\PCB\JAARK_PCB_MOTOR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C884B4F7-9A5B-4461-BD4E-20DECFB410DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6A063E-7635-4592-8FFA-48061525AD99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="9" windowWidth="22149" windowHeight="13920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JAARK_PCB_MOTOR" sheetId="1" r:id="rId1"/>
@@ -778,20 +778,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000030000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>This part is listed but is not stocked.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000031000000}">
+    <comment ref="J21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000030000000}">
       <text>
         <r>
           <rPr>
@@ -803,25 +790,29 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-  4000   $0.23    $935.76</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000032000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Desc: 45V 100MA 300MW TH TRANSISTOR-SM
-Footprint: TO-226-3, TO-92-3 (TO-226AA)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000033000000}">
+     1   $0.19      $0.19
+    10   $0.12      $1.19
+   100   $0.10     $10.41
+   500   $0.08     $38.30
+  1000   $0.07     $67.68</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000031000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Desc: TRANS PNP 40V 0.6A TO-92-3
+Footprint: TO-226-3, TO-92-3 (TO-226AA) Formed Leads</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000035000000}">
       <text>
         <r>
           <rPr>
@@ -844,7 +835,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000034000000}">
+    <comment ref="M22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000036000000}">
       <text>
         <r>
           <rPr>
@@ -863,7 +854,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000035000000}">
+    <comment ref="J23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000037000000}">
       <text>
         <r>
           <rPr>
@@ -886,7 +877,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000036000000}">
+    <comment ref="M23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000038000000}">
       <text>
         <r>
           <rPr>
@@ -905,7 +896,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000037000000}">
+    <comment ref="J24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000039000000}">
       <text>
         <r>
           <rPr>
@@ -928,7 +919,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000038000000}">
+    <comment ref="M24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003A000000}">
       <text>
         <r>
           <rPr>
@@ -947,7 +938,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000039000000}">
+    <comment ref="J25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003B000000}">
       <text>
         <r>
           <rPr>
@@ -966,7 +957,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003A000000}">
+    <comment ref="M25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003C000000}">
       <text>
         <r>
           <rPr>
@@ -985,7 +976,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003B000000}">
+    <comment ref="J26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003D000000}">
       <text>
         <r>
           <rPr>
@@ -1008,7 +999,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003C000000}">
+    <comment ref="M26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003E000000}">
       <text>
         <r>
           <rPr>
@@ -1027,7 +1018,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003D000000}">
+    <comment ref="J27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003F000000}">
       <text>
         <r>
           <rPr>
@@ -1039,27 +1030,32 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-     1   $0.63      $0.63
-    10   $0.47      $4.71
-    25   $0.42     $10.53
-   100   $0.38     $38.00</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003E000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Desc: FUSE CLIP BLADE 20A SMD</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00003F000000}">
+     1   $0.44      $0.44
+    10   $0.37      $3.70
+    25   $0.35      $8.66
+    50   $0.33     $16.49
+   100   $0.31     $31.41
+   250   $0.29     $73.59
+   500   $0.28    $140.14
+  1000   $0.27    $266.89
+  2500   $0.25    $625.42</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000040000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Desc: CONN RING CIRC 12-14AWG #6 CRIMP</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000041000000}">
       <text>
         <r>
           <rPr>
@@ -1072,7 +1068,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000040000000}">
+    <comment ref="I29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000042000000}">
       <text>
         <r>
           <rPr>
@@ -1085,7 +1081,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000041000000}">
+    <comment ref="F30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000043000000}">
       <text>
         <r>
           <rPr>
@@ -1103,7 +1099,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="92">
   <si>
     <t>Global Part Info</t>
   </si>
@@ -1186,7 +1182,7 @@
     <t>DRV8231DDAR</t>
   </si>
   <si>
-    <t>J1,J4-J6</t>
+    <t>J1,J4-J7</t>
   </si>
   <si>
     <t>1984617</t>
@@ -1210,16 +1206,13 @@
     <t>74438356018</t>
   </si>
   <si>
-    <t>Q1#1</t>
-  </si>
-  <si>
     <t>SSM3J334R</t>
   </si>
   <si>
-    <t>Q3</t>
-  </si>
-  <si>
-    <t>BC237B</t>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>2N4403TFR</t>
   </si>
   <si>
     <t>R1</t>
@@ -1255,7 +1248,7 @@
     <t>U1</t>
   </si>
   <si>
-    <t>3586TR</t>
+    <t>3568</t>
   </si>
   <si>
     <t>Digi-Key</t>
@@ -1318,7 +1311,7 @@
     <t>SSM3J334RLFCT-ND</t>
   </si>
   <si>
-    <t>1514-BC237BTREPBFREETR-ND</t>
+    <t>2N4403D26ZCT-ND</t>
   </si>
   <si>
     <t>A126350CT-ND</t>
@@ -1336,7 +1329,7 @@
     <t>RL12S.20FCT-ND</t>
   </si>
   <si>
-    <t>36-3586TRCT-ND</t>
+    <t>35684-ND</t>
   </si>
   <si>
     <t>Buy here</t>
@@ -1360,7 +1353,7 @@
     <t>Prj date:</t>
   </si>
   <si>
-    <t>2026-02-09 20:46:26 (file)</t>
+    <t>2026-02-15 16:47:53 (file)</t>
   </si>
   <si>
     <t>Board Qty:</t>
@@ -1375,21 +1368,20 @@
     <t>$ date:</t>
   </si>
   <si>
-    <t>2026-02-09 20:46:37</t>
+    <t>2026-02-15 16:48:51</t>
   </si>
   <si>
     <t>KiCost® v1.1.20</t>
   </si>
   <si>
-    <t xml:space="preserve">??? </t>
+    <t>Q1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.000"/>
   </numFmts>
@@ -1514,7 +1506,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1563,7 +1555,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1948,33 +1939,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr defaultRowHeight="14.6" outlineLevelCol="3" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="17.69140625" customWidth="1"/>
     <col min="2" max="2" width="11.69140625" customWidth="1"/>
     <col min="3" max="3" width="12.69140625" customWidth="1" outlineLevel="2"/>
-    <col min="4" max="4" width="20.69140625" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="9.15234375" outlineLevel="1"/>
+    <col min="4" max="4" width="23.921875" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="9.23046875" customWidth="1" outlineLevel="1"/>
     <col min="6" max="6" width="22.69140625" customWidth="1"/>
     <col min="7" max="7" width="16.69140625" customWidth="1"/>
     <col min="8" max="8" width="9.69140625" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="9.15234375" outlineLevel="2"/>
+    <col min="9" max="9" width="9.23046875" customWidth="1" outlineLevel="2"/>
     <col min="10" max="10" width="10.69140625" customWidth="1" outlineLevel="2"/>
-    <col min="11" max="11" width="0" hidden="1" customWidth="1" outlineLevel="3" collapsed="1"/>
+    <col min="11" max="11" width="9.23046875" customWidth="1" outlineLevel="3" collapsed="1"/>
     <col min="12" max="12" width="16.69140625" customWidth="1"/>
     <col min="13" max="13" width="26.69140625" customWidth="1" outlineLevel="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="F1" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G1" s="3">
         <v>1</v>
@@ -1982,34 +1973,34 @@
     </row>
     <row r="2" spans="1:13" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B2" s="2"/>
       <c r="F2" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G2" s="4">
         <f>TotalCost/BoardQty</f>
-        <v>20.420000000000005</v>
+        <v>19.260000000000009</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G3" s="5">
         <f>SUM(G7:G27)</f>
-        <v>20.420000000000005</v>
+        <v>19.260000000000009</v>
       </c>
       <c r="L3" s="5">
         <f>SUM(L7:L27)</f>
-        <v>18.400000000000006</v>
+        <v>19.260000000000009</v>
       </c>
       <c r="M3" s="6" t="str">
         <f>(COUNTA(L7:L27)&amp;" of "&amp;ROWS(L7:L27)&amp;" parts found")</f>
@@ -2018,10 +2009,10 @@
     </row>
     <row r="4" spans="1:13" ht="16.75" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18.45" x14ac:dyDescent="0.4">
@@ -2035,7 +2026,7 @@
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
       <c r="H5" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I5" s="15"/>
       <c r="J5" s="15"/>
@@ -2066,22 +2057,22 @@
         <v>7</v>
       </c>
       <c r="H6" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I6" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>53</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>6</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>7</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.4">
@@ -2125,7 +2116,7 @@
         <v>0.24</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.4">
@@ -2169,10 +2160,10 @@
         <v>0.15</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="29.15" x14ac:dyDescent="0.4">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="8" t="s">
         <v>13</v>
       </c>
@@ -2213,7 +2204,7 @@
         <v>0.4</v>
       </c>
       <c r="M9" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.4">
@@ -2257,10 +2248,10 @@
         <v>0.1</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="16.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="8" t="s">
         <v>17</v>
       </c>
@@ -2301,10 +2292,10 @@
         <v>0.41</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="29.15" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="14.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="8" t="s">
         <v>19</v>
       </c>
@@ -2345,7 +2336,7 @@
         <v>2.2599999999999998</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.4">
@@ -2365,15 +2356,16 @@
         <f>CEILING(BoardQty*1,1)</f>
         <v>1</v>
       </c>
-      <c r="F13" s="18">
-        <v>0.41</v>
-      </c>
-      <c r="G13" s="10">
+      <c r="F13" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G13" s="10" t="str">
         <f t="shared" si="1"/>
-        <v>0.41</v>
+        <v/>
       </c>
       <c r="H13" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I13" s="8"/>
       <c r="J13" s="9" t="str">
@@ -2388,7 +2380,7 @@
         <v/>
       </c>
       <c r="M13" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.4">
@@ -2432,7 +2424,7 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="M14" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.4">
@@ -2476,7 +2468,7 @@
         <v>3.02</v>
       </c>
       <c r="M15" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.4">
@@ -2493,8 +2485,8 @@
         <v>28</v>
       </c>
       <c r="E16" s="8">
-        <f>CEILING(BoardQty*4,1)</f>
-        <v>4</v>
+        <f>CEILING(BoardQty*5,1)</f>
+        <v>5</v>
       </c>
       <c r="F16" s="9">
         <f t="shared" si="0"/>
@@ -2502,7 +2494,7 @@
       </c>
       <c r="G16" s="10">
         <f t="shared" si="1"/>
-        <v>3.44</v>
+        <v>4.3</v>
       </c>
       <c r="H16" s="8">
         <v>12408</v>
@@ -2517,10 +2509,10 @@
       </c>
       <c r="L16" s="10">
         <f t="shared" si="2"/>
-        <v>3.44</v>
+        <v>4.3</v>
       </c>
       <c r="M16" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.4">
@@ -2549,7 +2541,7 @@
         <v>3.57</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I17" s="8"/>
       <c r="J17" s="9">
@@ -2564,7 +2556,7 @@
         <v>3.57</v>
       </c>
       <c r="M17" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.4">
@@ -2608,7 +2600,7 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="M18" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.4">
@@ -2652,21 +2644,21 @@
         <v>1.94</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A20" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>36</v>
       </c>
       <c r="E20" s="8">
         <f t="shared" si="3"/>
@@ -2696,64 +2688,65 @@
         <v>0.37</v>
       </c>
       <c r="M20" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A21" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>38</v>
       </c>
       <c r="E21" s="8">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="F21" s="9">
-        <v>1.61</v>
+        <f t="shared" si="0"/>
+        <v>0.19</v>
       </c>
       <c r="G21" s="10">
         <f t="shared" si="1"/>
-        <v>1.61</v>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>63</v>
+        <v>0.19</v>
+      </c>
+      <c r="H21" s="8">
+        <v>18574</v>
       </c>
       <c r="I21" s="8"/>
-      <c r="J21" s="9" t="str">
-        <f>IFERROR(IF(OR(I21&gt;=K21,E21&gt;=K21),LOOKUP(IF(I21="",E21,I21),{0,1,4000},{0,0.23394,0.23394}),"MOQ="&amp;K21),"")</f>
-        <v>MOQ=4000</v>
+      <c r="J21" s="9">
+        <f>IFERROR(IF(OR(I21&gt;=K21,E21&gt;=K21),LOOKUP(IF(I21="",E21,I21),{0,1,10,100,500,1000},{0,0.19,0.119,0.1041,0.0766,0.06768}),"MOQ="&amp;K21),"")</f>
+        <v>0.19</v>
       </c>
       <c r="K21" s="8">
-        <v>4000</v>
-      </c>
-      <c r="L21" s="10" t="str">
+        <v>1</v>
+      </c>
+      <c r="L21" s="10">
         <f t="shared" si="2"/>
-        <v/>
+        <v>0.19</v>
       </c>
       <c r="M21" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A22" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>39</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>40</v>
       </c>
       <c r="E22" s="8">
         <f t="shared" si="3"/>
@@ -2783,21 +2776,21 @@
         <v>0.1</v>
       </c>
       <c r="M22" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A23" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>41</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>42</v>
       </c>
       <c r="E23" s="8">
         <f t="shared" si="3"/>
@@ -2827,21 +2820,21 @@
         <v>0.1</v>
       </c>
       <c r="M23" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A24" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="E24" s="8">
         <f t="shared" si="3"/>
@@ -2871,21 +2864,21 @@
         <v>0.1</v>
       </c>
       <c r="M24" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A25" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>45</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>46</v>
       </c>
       <c r="E25" s="8">
         <f t="shared" si="3"/>
@@ -2915,21 +2908,21 @@
         <v>0.1</v>
       </c>
       <c r="M25" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A26" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>48</v>
       </c>
       <c r="E26" s="8">
         <f>CEILING(BoardQty*2,1)</f>
@@ -2959,21 +2952,21 @@
         <v>0.34</v>
       </c>
       <c r="M26" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A27" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>49</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>50</v>
       </c>
       <c r="E27" s="8">
         <f>CEILING(BoardQty*1,1)</f>
@@ -2981,41 +2974,41 @@
       </c>
       <c r="F27" s="9">
         <f t="shared" si="0"/>
-        <v>0.63</v>
+        <v>0.44</v>
       </c>
       <c r="G27" s="10">
         <f t="shared" si="1"/>
-        <v>0.63</v>
+        <v>0.44</v>
       </c>
       <c r="H27" s="8">
-        <v>54578</v>
+        <v>63044</v>
       </c>
       <c r="I27" s="8"/>
       <c r="J27" s="9">
-        <f>IFERROR(IF(OR(I27&gt;=K27,E27&gt;=K27),LOOKUP(IF(I27="",E27,I27),{0,1,10,25,100},{0,0.63,0.471,0.4212,0.38}),"MOQ="&amp;K27),"")</f>
-        <v>0.63</v>
+        <f>IFERROR(IF(OR(I27&gt;=K27,E27&gt;=K27),LOOKUP(IF(I27="",E27,I27),{0,1,10,25,50,100,250,500,1000,2500},{0,0.44,0.37,0.3464,0.3298,0.3141,0.29436,0.28028,0.26689,0.25017}),"MOQ="&amp;K27),"")</f>
+        <v>0.44</v>
       </c>
       <c r="K27" s="8">
         <v>1</v>
       </c>
       <c r="L27" s="10">
         <f t="shared" si="2"/>
-        <v>0.63</v>
+        <v>0.44</v>
       </c>
       <c r="M27" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="16.75" x14ac:dyDescent="0.4">
       <c r="F29" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G29" s="5">
         <f>SUM(L29)</f>
         <v>0</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I29" s="6" t="str">
         <f>IFERROR(IF(COUNTIF(I7:I27,"&gt;0")&gt;0,COUNTIF(I7:I27,"&gt;0")&amp;" of "&amp;(ROWS(K7:K27)-COUNTBLANK(K7:K27))&amp;" parts purchased",""),"")</f>
@@ -3028,13 +3021,13 @@
     </row>
     <row r="30" spans="1:13" ht="15.9" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I30" s="16" t="e">
-        <f>CONCATENATE(I53,I54,I55,I56,I57,I58,I59,I60,I61,I62,I63,I64,I65,I66,I67,I68,I69,I70,I71,I72,I73,I74)</f>
+        <f>CONCATENATE(I54,I55,I56,I57,I58,I59,I60,I61,I62,I63,I64,I65,I66,I67,I68,I69,I70,I71,I72,I73,I74,I75,I76)</f>
         <v>#N/A</v>
       </c>
       <c r="J30" s="17"/>
@@ -3174,18 +3167,19 @@
       <c r="L52" s="17"/>
     </row>
     <row r="53" spans="9:12" x14ac:dyDescent="0.4">
-      <c r="I53" t="str">
-        <f t="array" ref="I53:I74">IF(ISNUMBER(I7:I27)*(I7:I27&gt;=K7:K27)*(M7:M27&lt;&gt;""),TEXT(ROUNDUP(I7:I27/IF(ISNUMBER(K7:K27),K7:K27,1),0)*K7:K27,"##0")&amp;","&amp;M7:M27&amp;","&amp;SUBSTITUTE(SUBSTITUTE(IF(PURCHASE_DESCRIPTION&lt;&gt;"",PURCHASE_DESCRIPTION&amp;":","")&amp;A7:A27,",",";"),"
+      <c r="I53" s="17"/>
+      <c r="J53" s="17"/>
+      <c r="K53" s="17"/>
+      <c r="L53" s="17"/>
+    </row>
+    <row r="54" spans="9:12" x14ac:dyDescent="0.4">
+      <c r="I54" t="str">
+        <f t="array" ref="I54:I76">IF(ISNUMBER(I7:I27)*(I7:I27&gt;=K7:K27)*(M7:M27&lt;&gt;""),TEXT(ROUNDUP(I7:I27/IF(ISNUMBER(K7:K27),K7:K27,1),0)*K7:K27,"##0")&amp;","&amp;M7:M27&amp;","&amp;SUBSTITUTE(SUBSTITUTE(IF(PURCHASE_DESCRIPTION&lt;&gt;"",PURCHASE_DESCRIPTION&amp;":","")&amp;A7:A27,",",";"),"
 "," ")&amp;CHAR(10),"")</f>
         <v/>
       </c>
     </row>
-    <row r="54" spans="9:12" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="I54" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="9:12" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="9:12" x14ac:dyDescent="0.4">
       <c r="I55" t="str">
         <v/>
       </c>
@@ -3281,35 +3275,46 @@
       </c>
     </row>
     <row r="74" spans="9:9" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="I74" t="e">
+      <c r="I74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="9:9" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="I75" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="75" spans="9:9" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="76" spans="9:9" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="I76" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="77" spans="9:9" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="78" spans="9:9" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="H5:M5"/>
-    <mergeCell ref="I30:L52"/>
+    <mergeCell ref="I30:L53"/>
   </mergeCells>
   <conditionalFormatting sqref="E7:E9 E11:E27">
-    <cfRule type="cellIs" dxfId="8" priority="51" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="53" operator="greaterThan">
       <formula>SUM(IF(ISNUMBER(J7),I7,0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7:E27">
-    <cfRule type="expression" dxfId="7" priority="48">
+    <cfRule type="expression" dxfId="7" priority="50">
       <formula>AND(ISBLANK(D7),ISBLANK(L7))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="49">
+    <cfRule type="expression" dxfId="6" priority="51">
       <formula>IF(SUM(H7)=0,1,0)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="50" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="52" operator="greaterThan">
       <formula>SUM(H7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="cellIs" dxfId="4" priority="63" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="65" operator="greaterThan">
       <formula>SUM(IF(ISNUMBER(J10),I10,0))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3323,7 +3328,7 @@
       <formula>AND(NOT(ISBLANK(I7)),OR(H7="NonStk",I7&gt;H7))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I13 I21">
+  <conditionalFormatting sqref="I13">
     <cfRule type="expression" dxfId="1" priority="14">
       <formula>AND(I13&gt;0,MOD(I13,K13)&lt;&gt;0)</formula>
     </cfRule>
@@ -3357,22 +3362,23 @@
     <hyperlink ref="M19" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
     <hyperlink ref="D20" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
     <hyperlink ref="M20" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="M21" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="D22" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="M22" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="D23" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="M23" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="D24" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="M24" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="D25" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="M25" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="D26" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="M26" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="D27" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="M27" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="H29" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="D21" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="M21" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="D22" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="M22" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="D23" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="M23" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="D24" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="M24" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="D25" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="M25" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="D26" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="M26" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="D27" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="M27" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="H29" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId38"/>
+  <legacyDrawing r:id="rId39"/>
 </worksheet>
 </file>
</xml_diff>